<commit_message>
actualizacion exdel con obras
actualizacion exdel con obras
</commit_message>
<xml_diff>
--- a/obras.xlsx
+++ b/obras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mfournier\Pictures\2026\web-new\manuel_fournier_web_github_pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F988F3B8-2783-4962-A847-EBF5727DA3B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9D8784-363A-45E6-A910-3F06034550E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -613,7 +613,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -633,7 +633,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>